<commit_message>
fix(tools): bound fiscal dates and reject invalid workbook periods
</commit_message>
<xml_diff>
--- a/public/downloads/modele-rapprochement-bancaire.xlsx
+++ b/public/downloads/modele-rapprochement-bancaire.xlsx
@@ -511,7 +511,7 @@
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>B5/B6 : période du contrôle. B8/B9 : soldes à la même date de fin.</t>
+          <t>B5/B6 : dates entières du 01/01/1900 au 31/12/9999 (système Excel 1900, faux 29/02/1900 exclu). B8/B9 : soldes à la même date de fin.</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
         </is>
       </c>
       <c r="B24" s="6">
-        <f>IFERROR(IF(COUNT(B5:B6,B8:B9,B11:B12,B14:B15,B17)&lt;&gt;9,"NON VALIDÉ — saisie incomplète",IF(OR(ABS(B8)&gt;999999999.99,ROUND(B8,2)&lt;&gt;B8,ABS(B9)&gt;999999999.99,ROUND(B9,2)&lt;&gt;B9,ABS(B11)&gt;999999999.99,ROUND(B11,2)&lt;&gt;B11,ABS(B12)&gt;999999999.99,ROUND(B12,2)&lt;&gt;B12,ABS(B14)&gt;999999999.99,ROUND(B14,2)&lt;&gt;B14,ABS(B15)&gt;999999999.99,ROUND(B15,2)&lt;&gt;B15,ABS(B17)&gt;999999999.99,ROUND(B17,2)&lt;&gt;B17),"NON VALIDÉ — montant hors borne ou précision",IF(B5&gt;B6,"NON VALIDÉ — période inversée",IF(OR(B17&lt;&gt;0,B22&lt;&gt;0),"NON VALIDÉ — écart à expliquer","Soldes concordants — à valider")))),"NON VALIDÉ — saisie invalide")</f>
+        <f>IFERROR(IF(OR(NOT(ISNUMBER(B5)),B5&lt;1,B5&gt;2958465,INT(B5)&lt;&gt;B5,B5=60,NOT(ISNUMBER(B6)),B6&lt;1,B6&gt;2958465,INT(B6)&lt;&gt;B6,B6=60),"NON VALIDÉ — date hors borne ou invalide",IF(COUNT(B5:B6,B8:B9,B11:B12,B14:B15,B17)&lt;&gt;9,"NON VALIDÉ — saisie incomplète",IF(OR(ABS(B8)&gt;999999999.99,ROUND(B8,2)&lt;&gt;B8,ABS(B9)&gt;999999999.99,ROUND(B9,2)&lt;&gt;B9,ABS(B11)&gt;999999999.99,ROUND(B11,2)&lt;&gt;B11,ABS(B12)&gt;999999999.99,ROUND(B12,2)&lt;&gt;B12,ABS(B14)&gt;999999999.99,ROUND(B14,2)&lt;&gt;B14,ABS(B15)&gt;999999999.99,ROUND(B15,2)&lt;&gt;B15,ABS(B17)&gt;999999999.99,ROUND(B17,2)&lt;&gt;B17),"NON VALIDÉ — montant hors borne ou précision",IF(B5&gt;B6,"NON VALIDÉ — période inversée",IF(OR(B17&lt;&gt;0,B22&lt;&gt;0),"NON VALIDÉ — écart à expliquer","Soldes concordants — à valider"))))),"NON VALIDÉ — saisie invalide")</f>
         <v/>
       </c>
       <c r="C24" s="2" t="n"/>
@@ -1282,7 +1282,7 @@
         </is>
       </c>
       <c r="B24" s="6">
-        <f>IFERROR(IF(COUNT(B5:B6,B8:B9,B11:B12,B14:B15,B17)&lt;&gt;9,"NON VALIDÉ — saisie incomplète",IF(OR(ABS(B8)&gt;999999999.99,ROUND(B8,2)&lt;&gt;B8,ABS(B9)&gt;999999999.99,ROUND(B9,2)&lt;&gt;B9,ABS(B11)&gt;999999999.99,ROUND(B11,2)&lt;&gt;B11,ABS(B12)&gt;999999999.99,ROUND(B12,2)&lt;&gt;B12,ABS(B14)&gt;999999999.99,ROUND(B14,2)&lt;&gt;B14,ABS(B15)&gt;999999999.99,ROUND(B15,2)&lt;&gt;B15,ABS(B17)&gt;999999999.99,ROUND(B17,2)&lt;&gt;B17),"NON VALIDÉ — montant hors borne ou précision",IF(B5&gt;B6,"NON VALIDÉ — période inversée",IF(OR(B17&lt;&gt;0,B22&lt;&gt;0),"NON VALIDÉ — écart à expliquer","Soldes concordants — à valider")))),"NON VALIDÉ — saisie invalide")</f>
+        <f>IFERROR(IF(OR(NOT(ISNUMBER(B5)),B5&lt;1,B5&gt;2958465,INT(B5)&lt;&gt;B5,B5=60,NOT(ISNUMBER(B6)),B6&lt;1,B6&gt;2958465,INT(B6)&lt;&gt;B6,B6=60),"NON VALIDÉ — date hors borne ou invalide",IF(COUNT(B5:B6,B8:B9,B11:B12,B14:B15,B17)&lt;&gt;9,"NON VALIDÉ — saisie incomplète",IF(OR(ABS(B8)&gt;999999999.99,ROUND(B8,2)&lt;&gt;B8,ABS(B9)&gt;999999999.99,ROUND(B9,2)&lt;&gt;B9,ABS(B11)&gt;999999999.99,ROUND(B11,2)&lt;&gt;B11,ABS(B12)&gt;999999999.99,ROUND(B12,2)&lt;&gt;B12,ABS(B14)&gt;999999999.99,ROUND(B14,2)&lt;&gt;B14,ABS(B15)&gt;999999999.99,ROUND(B15,2)&lt;&gt;B15,ABS(B17)&gt;999999999.99,ROUND(B17,2)&lt;&gt;B17),"NON VALIDÉ — montant hors borne ou précision",IF(B5&gt;B6,"NON VALIDÉ — période inversée",IF(OR(B17&lt;&gt;0,B22&lt;&gt;0),"NON VALIDÉ — écart à expliquer","Soldes concordants — à valider"))))),"NON VALIDÉ — saisie invalide")</f>
         <v/>
       </c>
       <c r="C24" s="2" t="n"/>

</xml_diff>